<commit_message>
Phase 2 Part : Create Bypass in Decode/Execute/Memory Stages for rs_data/rt_data
</commit_message>
<xml_diff>
--- a/docs/MIPS I ISA.xlsx
+++ b/docs/MIPS I ISA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Digital\SoC\mips_top\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2371D3D4-A0C2-4C68-8323-3F3C1DAB6AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81237FEF-D802-4B88-8411-040CA84ACE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main ISA" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="452">
   <si>
     <t xml:space="preserve">Opcode </t>
   </si>
@@ -1366,6 +1366,60 @@
   </si>
   <si>
     <t>Unsigned division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Execute </t>
+  </si>
+  <si>
+    <t>Memory</t>
+  </si>
+  <si>
+    <t>Writeback</t>
+  </si>
+  <si>
+    <t>Control Hazard</t>
+  </si>
+  <si>
+    <t>Data Hazard</t>
+  </si>
+  <si>
+    <t>Branch</t>
+  </si>
+  <si>
+    <t>Flush f2d register</t>
+  </si>
+  <si>
+    <t>Flush f2d register +handle $ra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used </t>
+  </si>
+  <si>
+    <t>Used</t>
+  </si>
+  <si>
+    <t>Memory/WB 2 Execute Bypass</t>
+  </si>
+  <si>
+    <t>Stall</t>
+  </si>
+  <si>
+    <t>WB 2 Memory Bypass</t>
+  </si>
+  <si>
+    <t>Early Detection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch Hazards </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Jump Hazards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">handled in Decode Stage </t>
+  </si>
+  <si>
+    <t>Execute/Memory/WB 2 Decode Bypass</t>
   </si>
 </sst>
 </file>
@@ -1415,7 +1469,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1456,6 +1510,18 @@
       <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1540,7 +1606,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1602,11 +1668,157 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="49">
+  <dxfs count="59">
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -1722,120 +1934,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1993,8 +2091,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}" name="Table1" displayName="Table1" ref="A1:T32" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47">
-  <autoFilter ref="A1:T32" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}" name="Table1" displayName="Table1" ref="A1:Y32" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
+  <autoFilter ref="A1:Y32" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}">
     <filterColumn colId="4">
       <filters>
         <filter val="[DONE] Phase 1 - Assignement 1"/>
@@ -2003,35 +2101,40 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{6F141741-2C51-4220-AFC7-E5871EC6CD8F}" name="Opcode " dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{94AD8F24-8B7B-488A-B2A5-515BD41E7F08}" name="Name " dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{F54D0553-BC6A-48B5-9E0F-A0BF767398A8}" name="Description " dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{E6BC317F-8DC6-4A10-97A3-062D0A6033C4}" name="Operation" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{4C0751C6-22DE-48F3-A333-C0824C0F0EFD}" name="Comments" dataDxfId="42"/>
-    <tableColumn id="6" xr3:uid="{599EA1B7-5FC4-4650-9D00-5A65D2D76FD2}" name="ReWrite" dataDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{FADF9286-B678-4102-91DC-1ADDBF050E85}" name="RegDst" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{0CF239B5-36C7-4DBC-8249-487AE1E5F5A5}" name="AluSrc" dataDxfId="39"/>
-    <tableColumn id="9" xr3:uid="{1BC2ABDC-0C79-4111-A3DE-6C63C94FA5D5}" name="MemWrite" dataDxfId="38"/>
-    <tableColumn id="10" xr3:uid="{0153894A-151B-41AD-B603-B7BF55EEBE9C}" name="Write_back_sel" dataDxfId="37"/>
-    <tableColumn id="11" xr3:uid="{C68ADF0D-C375-4115-93EF-CD4021B0BD3E}" name="AluOp" dataDxfId="36"/>
+  <tableColumns count="25">
+    <tableColumn id="1" xr3:uid="{6F141741-2C51-4220-AFC7-E5871EC6CD8F}" name="Opcode " dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{94AD8F24-8B7B-488A-B2A5-515BD41E7F08}" name="Name " dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{F54D0553-BC6A-48B5-9E0F-A0BF767398A8}" name="Description " dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{E6BC317F-8DC6-4A10-97A3-062D0A6033C4}" name="Operation" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{4C0751C6-22DE-48F3-A333-C0824C0F0EFD}" name="Comments" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{599EA1B7-5FC4-4650-9D00-5A65D2D76FD2}" name="ReWrite" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{FADF9286-B678-4102-91DC-1ADDBF050E85}" name="RegDst" dataDxfId="39"/>
+    <tableColumn id="8" xr3:uid="{0CF239B5-36C7-4DBC-8249-487AE1E5F5A5}" name="AluSrc" dataDxfId="38"/>
+    <tableColumn id="9" xr3:uid="{1BC2ABDC-0C79-4111-A3DE-6C63C94FA5D5}" name="MemWrite" dataDxfId="37"/>
+    <tableColumn id="10" xr3:uid="{0153894A-151B-41AD-B603-B7BF55EEBE9C}" name="Write_back_sel" dataDxfId="36"/>
+    <tableColumn id="11" xr3:uid="{C68ADF0D-C375-4115-93EF-CD4021B0BD3E}" name="AluOp" dataDxfId="35"/>
     <tableColumn id="20" xr3:uid="{4B7A4639-28F0-4297-B746-1FB610AB5BC3}" name="AluOp_immediate"/>
     <tableColumn id="18" xr3:uid="{8FFAE8F4-2929-40DB-8CDB-B6B62F5A5B1D}" name="wb_se_select"/>
     <tableColumn id="21" xr3:uid="{83AF33B5-363D-492B-8E5C-C63E2DB98A90}" name="se_select"/>
-    <tableColumn id="12" xr3:uid="{F1D4D373-D3C9-4BF4-9941-4766A9F778CF}" name="Overflow Mask" dataDxfId="35"/>
-    <tableColumn id="13" xr3:uid="{E4CE9616-85BB-465A-8E96-A5EC285FC9E7}" name="PC Src" dataDxfId="34"/>
-    <tableColumn id="14" xr3:uid="{65386F80-7AF9-4CF2-BDE0-29D2094B577A}" name="hi_write" dataDxfId="33"/>
-    <tableColumn id="15" xr3:uid="{FA558C62-1F5B-4CE1-A1DE-149585FE9142}" name="lo_write" dataDxfId="32"/>
-    <tableColumn id="16" xr3:uid="{D1B88377-9E5B-4D25-B01D-35C955F02CF0}" name="hi_select" dataDxfId="31"/>
-    <tableColumn id="17" xr3:uid="{F28DE1E5-F9D3-44FC-AA82-3DBE9E42FAEC}" name="lo_select" dataDxfId="30"/>
+    <tableColumn id="12" xr3:uid="{F1D4D373-D3C9-4BF4-9941-4766A9F778CF}" name="Overflow Mask" dataDxfId="34"/>
+    <tableColumn id="13" xr3:uid="{E4CE9616-85BB-465A-8E96-A5EC285FC9E7}" name="PC Src" dataDxfId="33"/>
+    <tableColumn id="14" xr3:uid="{65386F80-7AF9-4CF2-BDE0-29D2094B577A}" name="hi_write" dataDxfId="32"/>
+    <tableColumn id="15" xr3:uid="{FA558C62-1F5B-4CE1-A1DE-149585FE9142}" name="lo_write" dataDxfId="31"/>
+    <tableColumn id="16" xr3:uid="{D1B88377-9E5B-4D25-B01D-35C955F02CF0}" name="hi_select" dataDxfId="30"/>
+    <tableColumn id="17" xr3:uid="{F28DE1E5-F9D3-44FC-AA82-3DBE9E42FAEC}" name="lo_select" dataDxfId="29"/>
+    <tableColumn id="19" xr3:uid="{390BDAAC-6935-4C11-B3D2-24BF002BA904}" name="Execute " dataDxfId="4"/>
+    <tableColumn id="22" xr3:uid="{D9F15294-478E-42F4-BA78-FA287163229E}" name="Memory" dataDxfId="3"/>
+    <tableColumn id="23" xr3:uid="{FF7FA640-5713-4F28-BCA2-FA75BE7EA342}" name="Writeback" dataDxfId="2"/>
+    <tableColumn id="24" xr3:uid="{959B7067-1726-4B40-95D5-DFB8C3638973}" name="Control Hazard" dataDxfId="1"/>
+    <tableColumn id="25" xr3:uid="{D22C01B1-0878-4B6A-95B0-C87FF0D4AE43}" name="Data Hazard" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}" name="Table2" displayName="Table2" ref="A1:Q29" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
-  <autoFilter ref="A1:Q29" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}" name="Table2" displayName="Table2" ref="A1:V29" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+  <autoFilter ref="A1:V29" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}">
     <filterColumn colId="4">
       <filters>
         <filter val="[DONE] Phase 1 - Assignement 1"/>
@@ -2041,49 +2144,54 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{CD4B495D-BEBD-4687-9E48-13E31F1A5458}" name="Funct " dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{E7F73B4A-D35B-4A89-BCB0-DFA47DFF3033}" name="Name " dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{87DDDCA8-8D3D-45D9-835E-8024A1DEE513}" name="Description " dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{1A74FB59-C961-44A8-A91C-BB37DF112620}" name="Operation" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{916118AB-C4A0-47F3-87B2-8F2F5A96272D}" name="Comments" dataDxfId="23"/>
-    <tableColumn id="12" xr3:uid="{A9D2244B-08FE-4D9B-B85E-939B8D1FCDA2}" name="ReWrite" dataDxfId="22"/>
-    <tableColumn id="13" xr3:uid="{0B472683-72C5-483F-A1F5-D2FDA9886CAC}" name="RegDst" dataDxfId="21"/>
-    <tableColumn id="14" xr3:uid="{B2AB814A-4427-483D-92F7-16C5C8659619}" name="AluSrc" dataDxfId="20"/>
-    <tableColumn id="16" xr3:uid="{D1503AC1-DA6F-431E-86E3-3CD8BAD27F47}" name="Write_Back_sel" dataDxfId="19"/>
-    <tableColumn id="17" xr3:uid="{03DAA7C4-6940-4324-93F3-3F703363AC9E}" name="AluOp" dataDxfId="18"/>
-    <tableColumn id="18" xr3:uid="{B4769B34-7E40-48A1-81CF-AF31CD8F17DF}" name="overflow Mask" dataDxfId="17"/>
-    <tableColumn id="19" xr3:uid="{804568FB-85BF-40E3-B057-9BD0161489CA}" name="PCsrc" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{E7BF6538-000F-4221-BEAF-1B1069F544DF}" name="hi_write" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{EB15F963-101B-4FD6-8C35-479C603DBCE6}" name="lo_write" dataDxfId="14"/>
-    <tableColumn id="10" xr3:uid="{B96C025F-6BE7-4A63-8A28-B9122951D973}" name="hi_select" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{585ED190-3E47-430F-B835-ADAC4874BFFD}" name="lo_select" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{2C2B3870-9B9E-459D-B78A-1F301F881E15}" name="AluControl" dataDxfId="11"/>
+  <tableColumns count="22">
+    <tableColumn id="1" xr3:uid="{CD4B495D-BEBD-4687-9E48-13E31F1A5458}" name="Funct " dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{E7F73B4A-D35B-4A89-BCB0-DFA47DFF3033}" name="Name " dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{87DDDCA8-8D3D-45D9-835E-8024A1DEE513}" name="Description " dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{1A74FB59-C961-44A8-A91C-BB37DF112620}" name="Operation" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{916118AB-C4A0-47F3-87B2-8F2F5A96272D}" name="Comments" dataDxfId="22"/>
+    <tableColumn id="12" xr3:uid="{A9D2244B-08FE-4D9B-B85E-939B8D1FCDA2}" name="ReWrite" dataDxfId="21"/>
+    <tableColumn id="13" xr3:uid="{0B472683-72C5-483F-A1F5-D2FDA9886CAC}" name="RegDst" dataDxfId="20"/>
+    <tableColumn id="14" xr3:uid="{B2AB814A-4427-483D-92F7-16C5C8659619}" name="AluSrc" dataDxfId="19"/>
+    <tableColumn id="16" xr3:uid="{D1503AC1-DA6F-431E-86E3-3CD8BAD27F47}" name="Write_Back_sel" dataDxfId="18"/>
+    <tableColumn id="17" xr3:uid="{03DAA7C4-6940-4324-93F3-3F703363AC9E}" name="AluOp" dataDxfId="17"/>
+    <tableColumn id="18" xr3:uid="{B4769B34-7E40-48A1-81CF-AF31CD8F17DF}" name="overflow Mask" dataDxfId="16"/>
+    <tableColumn id="19" xr3:uid="{804568FB-85BF-40E3-B057-9BD0161489CA}" name="PCsrc" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{E7BF6538-000F-4221-BEAF-1B1069F544DF}" name="hi_write" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{EB15F963-101B-4FD6-8C35-479C603DBCE6}" name="lo_write" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{B96C025F-6BE7-4A63-8A28-B9122951D973}" name="hi_select" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{585ED190-3E47-430F-B835-ADAC4874BFFD}" name="lo_select" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{2C2B3870-9B9E-459D-B78A-1F301F881E15}" name="AluControl" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{6F7BBD8D-8BB1-43BB-92F8-BA3005A4DF49}" name="Execute " dataDxfId="9"/>
+    <tableColumn id="15" xr3:uid="{1FF65792-45A2-40C0-8B41-9DB94001A189}" name="Memory" dataDxfId="8"/>
+    <tableColumn id="20" xr3:uid="{5E12103B-CEA1-489E-B3A0-711EF959001C}" name="Writeback" dataDxfId="7"/>
+    <tableColumn id="21" xr3:uid="{9DFD91F3-7DF9-46A0-9289-D1240309AAF3}" name="Control Hazard" dataDxfId="6"/>
+    <tableColumn id="22" xr3:uid="{8AA0B39B-B245-4D8F-97FF-7A4FD54C1E29}" name="Data Hazard" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D53E060B-7B9B-43C9-B6C3-0ADAD9EBE1D7}" name="Table3" displayName="Table3" ref="A1:D10" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D53E060B-7B9B-43C9-B6C3-0ADAD9EBE1D7}" name="Table3" displayName="Table3" ref="A1:D10" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="A1:D10" xr:uid="{D53E060B-7B9B-43C9-B6C3-0ADAD9EBE1D7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{9277D667-9F6C-4B1A-9BD6-8F4F09DC6FCC}" name="Funct " dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{44121D79-0FB6-4BA0-822D-A22356C92E27}" name="Name " dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{9FFE180B-8031-4716-9450-AF517E4275A8}" name="Description " dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{700AEF16-A70F-499B-87D2-32234302488E}" name="Operation" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{9277D667-9F6C-4B1A-9BD6-8F4F09DC6FCC}" name="Funct " dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{44121D79-0FB6-4BA0-822D-A22356C92E27}" name="Name " dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{9FFE180B-8031-4716-9450-AF517E4275A8}" name="Description " dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{700AEF16-A70F-499B-87D2-32234302488E}" name="Operation" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4ED1B589-2AD4-4E0A-A923-4EE6DF5E917F}" name="Table4" displayName="Table4" ref="A1:C11" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4ED1B589-2AD4-4E0A-A923-4EE6DF5E917F}" name="Table4" displayName="Table4" ref="A1:C11" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
   <autoFilter ref="A1:C11" xr:uid="{4ED1B589-2AD4-4E0A-A923-4EE6DF5E917F}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{54084E4B-9E28-4AC8-AF1B-3C8B1A6C439F}" name="Test #" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{BD73A61D-1FF1-4476-B2A3-42E28CFEB520}" name="Function" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{89ABFDA6-6F2C-4281-BB66-65F42B941C05}" name="Description" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{54084E4B-9E28-4AC8-AF1B-3C8B1A6C439F}" name="Test #" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{BD73A61D-1FF1-4476-B2A3-42E28CFEB520}" name="Function" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{89ABFDA6-6F2C-4281-BB66-65F42B941C05}" name="Description" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2352,21 +2460,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T32"/>
+  <dimension ref="A1:AB32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="20.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.6640625" customWidth="1"/>
     <col min="4" max="4" width="32.5546875" customWidth="1"/>
     <col min="5" max="5" width="36.5546875" customWidth="1"/>
+    <col min="6" max="9" width="8.88671875" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="8.88671875" customWidth="1"/>
     <col min="12" max="13" width="14.21875" customWidth="1"/>
-    <col min="15" max="15" width="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.88671875" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="16" width="17.33203125" customWidth="1"/>
+    <col min="17" max="20" width="8.88671875" customWidth="1"/>
+    <col min="24" max="24" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2427,8 +2544,29 @@
       <c r="T1" s="16" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+      <c r="U1" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="AA1" s="21" t="s">
+        <v>448</v>
+      </c>
+      <c r="AB1" s="22" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2447,7 +2585,7 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
     </row>
-    <row r="3" spans="1:20" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>90</v>
       </c>
@@ -2488,8 +2626,20 @@
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="X3" t="s">
+        <v>439</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>451</v>
+      </c>
+      <c r="AA3" s="21" t="s">
+        <v>449</v>
+      </c>
+      <c r="AB3" s="22" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -2512,8 +2662,11 @@
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
       <c r="T4" s="1"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="X4" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -2554,8 +2707,11 @@
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="X5" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -2593,8 +2749,14 @@
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="X6" t="s">
+        <v>439</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
@@ -2635,8 +2797,14 @@
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="X7" t="s">
+        <v>439</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
@@ -2677,8 +2845,14 @@
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="X8" t="s">
+        <v>439</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
@@ -2719,8 +2893,14 @@
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
       <c r="T9" s="1"/>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="X9" t="s">
+        <v>439</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>32</v>
       </c>
@@ -2764,8 +2944,17 @@
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
       <c r="T10" s="1"/>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U10" t="s">
+        <v>442</v>
+      </c>
+      <c r="W10" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>36</v>
       </c>
@@ -2788,8 +2977,17 @@
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U11" t="s">
+        <v>442</v>
+      </c>
+      <c r="W11" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>39</v>
       </c>
@@ -2833,8 +3031,17 @@
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U12" t="s">
+        <v>442</v>
+      </c>
+      <c r="W12" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>43</v>
       </c>
@@ -2854,8 +3061,17 @@
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U13" t="s">
+        <v>442</v>
+      </c>
+      <c r="W13" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>46</v>
       </c>
@@ -2899,8 +3115,17 @@
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U14" t="s">
+        <v>442</v>
+      </c>
+      <c r="W14" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>50</v>
       </c>
@@ -2944,8 +3169,17 @@
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U15" t="s">
+        <v>442</v>
+      </c>
+      <c r="W15" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>54</v>
       </c>
@@ -2989,8 +3223,17 @@
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U16" t="s">
+        <v>442</v>
+      </c>
+      <c r="W16" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>58</v>
       </c>
@@ -3022,8 +3265,17 @@
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
-    </row>
-    <row r="18" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="U17" t="s">
+        <v>442</v>
+      </c>
+      <c r="W17" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>94</v>
       </c>
@@ -3044,7 +3296,7 @@
       <c r="S18" s="1"/>
       <c r="T18" s="1"/>
     </row>
-    <row r="19" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>63</v>
       </c>
@@ -3063,7 +3315,7 @@
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
     </row>
-    <row r="20" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:25" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>98</v>
       </c>
@@ -3082,7 +3334,7 @@
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
     </row>
-    <row r="21" spans="1:20" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>97</v>
       </c>
@@ -3111,8 +3363,17 @@
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U21" t="s">
+        <v>442</v>
+      </c>
+      <c r="W21" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>70</v>
       </c>
@@ -3153,8 +3414,17 @@
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
       <c r="T22" s="1"/>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V22" t="s">
+        <v>443</v>
+      </c>
+      <c r="W22" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>74</v>
       </c>
@@ -3195,8 +3465,17 @@
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V23" t="s">
+        <v>443</v>
+      </c>
+      <c r="W23" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>78</v>
       </c>
@@ -3234,8 +3513,17 @@
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V24" t="s">
+        <v>443</v>
+      </c>
+      <c r="W24" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>82</v>
       </c>
@@ -3276,8 +3564,17 @@
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V25" t="s">
+        <v>443</v>
+      </c>
+      <c r="W25" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>86</v>
       </c>
@@ -3318,8 +3615,17 @@
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
       <c r="T26" s="1"/>
-    </row>
-    <row r="27" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+      <c r="V26" t="s">
+        <v>443</v>
+      </c>
+      <c r="W26" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>102</v>
       </c>
@@ -3340,7 +3646,7 @@
       <c r="S27" s="1"/>
       <c r="T27" s="1"/>
     </row>
-    <row r="28" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>106</v>
       </c>
@@ -3361,7 +3667,7 @@
       <c r="S28" s="1"/>
       <c r="T28" s="1"/>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>110</v>
       </c>
@@ -3399,8 +3705,14 @@
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
-    </row>
-    <row r="30" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+      <c r="V29" t="s">
+        <v>443</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>114</v>
       </c>
@@ -3419,7 +3731,7 @@
       <c r="S30" s="1"/>
       <c r="T30" s="1"/>
     </row>
-    <row r="31" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>118</v>
       </c>
@@ -3438,7 +3750,7 @@
       <c r="S31" s="1"/>
       <c r="T31" s="1"/>
     </row>
-    <row r="32" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -3469,22 +3781,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8344681D-13F5-4AA9-8C1C-9376E6ED3191}">
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:V32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
     <col min="2" max="2" width="21.109375" customWidth="1"/>
     <col min="3" max="5" width="28.44140625" customWidth="1"/>
-    <col min="9" max="9" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="8.88671875" customWidth="1"/>
+    <col min="9" max="9" width="16.109375" customWidth="1"/>
+    <col min="10" max="10" width="8.88671875" customWidth="1"/>
+    <col min="11" max="11" width="15.77734375" customWidth="1"/>
+    <col min="12" max="12" width="8.88671875" customWidth="1"/>
     <col min="13" max="13" width="10.21875" customWidth="1"/>
     <col min="14" max="14" width="12.6640625" customWidth="1"/>
     <col min="15" max="15" width="11.77734375" customWidth="1"/>
     <col min="16" max="16" width="12.109375" customWidth="1"/>
     <col min="17" max="17" width="20.109375" customWidth="1"/>
+    <col min="21" max="21" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="26.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>122</v>
       </c>
@@ -3536,8 +3853,23 @@
       <c r="Q1" s="1" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R1" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -3575,8 +3907,17 @@
       <c r="Q2" s="1" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R2" t="s">
+        <v>442</v>
+      </c>
+      <c r="T2" t="s">
+        <v>443</v>
+      </c>
+      <c r="V2" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -3614,8 +3955,17 @@
       <c r="Q3" s="1" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R3" t="s">
+        <v>442</v>
+      </c>
+      <c r="T3" t="s">
+        <v>443</v>
+      </c>
+      <c r="V3" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -3653,8 +4003,17 @@
       <c r="Q4" s="1" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R4" t="s">
+        <v>442</v>
+      </c>
+      <c r="T4" t="s">
+        <v>443</v>
+      </c>
+      <c r="V4" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -3692,8 +4051,17 @@
       <c r="Q5" s="1" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R5" t="s">
+        <v>442</v>
+      </c>
+      <c r="T5" t="s">
+        <v>443</v>
+      </c>
+      <c r="V5" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -3731,8 +4099,17 @@
       <c r="Q6" s="1" t="s">
         <v>320</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R6" t="s">
+        <v>442</v>
+      </c>
+      <c r="T6" t="s">
+        <v>443</v>
+      </c>
+      <c r="V6" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -3770,8 +4147,17 @@
       <c r="Q7" s="1" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R7" t="s">
+        <v>442</v>
+      </c>
+      <c r="T7" t="s">
+        <v>443</v>
+      </c>
+      <c r="V7" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>32</v>
       </c>
@@ -3811,8 +4197,15 @@
       <c r="Q8" s="1" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" t="s">
+        <v>440</v>
+      </c>
+      <c r="V8" s="1"/>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
@@ -3862,8 +4255,15 @@
       <c r="Q9" s="1" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="1"/>
+      <c r="U9" t="s">
+        <v>441</v>
+      </c>
+      <c r="V9" s="1"/>
+    </row>
+    <row r="10" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>145</v>
       </c>
@@ -3891,8 +4291,13 @@
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
-    </row>
-    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="R10" s="1"/>
+      <c r="S10" s="1"/>
+      <c r="T10" s="1"/>
+      <c r="U10" s="1"/>
+      <c r="V10" s="1"/>
+    </row>
+    <row r="11" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>149</v>
       </c>
@@ -3920,8 +4325,13 @@
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R11" s="1"/>
+      <c r="S11" s="1"/>
+      <c r="T11" s="1"/>
+      <c r="U11" s="1"/>
+      <c r="V11" s="1"/>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>152</v>
       </c>
@@ -3969,8 +4379,17 @@
       <c r="Q12" s="1" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R12" s="1"/>
+      <c r="S12" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="T12" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U12" s="1"/>
+      <c r="V12" s="1"/>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>63</v>
       </c>
@@ -4018,8 +4437,17 @@
       <c r="Q13" s="1" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R13" s="1"/>
+      <c r="S13" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="T13" s="1"/>
+      <c r="U13" s="1"/>
+      <c r="V13" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>159</v>
       </c>
@@ -4067,8 +4495,17 @@
       <c r="Q14" s="1" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R14" s="1"/>
+      <c r="S14" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="T14" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U14" s="1"/>
+      <c r="V14" s="1"/>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>163</v>
       </c>
@@ -4116,8 +4553,17 @@
       <c r="Q15" s="1" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R15" s="1"/>
+      <c r="S15" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+      <c r="V15" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>167</v>
       </c>
@@ -4155,8 +4601,19 @@
         <v>329</v>
       </c>
       <c r="Q16" s="1"/>
-    </row>
-    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+      <c r="R16" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S16" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+      <c r="V16" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>171</v>
       </c>
@@ -4182,8 +4639,13 @@
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
-    </row>
-    <row r="18" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
+      <c r="T17" s="1"/>
+      <c r="U17" s="1"/>
+      <c r="V17" s="1"/>
+    </row>
+    <row r="18" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>174</v>
       </c>
@@ -4221,8 +4683,19 @@
         <v>304</v>
       </c>
       <c r="Q18" s="1"/>
-    </row>
-    <row r="19" spans="1:17" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="R18" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S18" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="T18" s="1"/>
+      <c r="U18" s="1"/>
+      <c r="V18" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>177</v>
       </c>
@@ -4248,8 +4721,13 @@
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="1"/>
+      <c r="U19" s="1"/>
+      <c r="V19" s="1"/>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>70</v>
       </c>
@@ -4290,8 +4768,19 @@
       <c r="Q20" s="1" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R20" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S20" s="1"/>
+      <c r="T20" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U20" s="1"/>
+      <c r="V20" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>74</v>
       </c>
@@ -4321,8 +4810,19 @@
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R21" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S21" s="1"/>
+      <c r="T21" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U21" s="1"/>
+      <c r="V21" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>185</v>
       </c>
@@ -4363,8 +4863,19 @@
       <c r="Q22" s="1" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R22" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S22" s="1"/>
+      <c r="T22" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U22" s="1"/>
+      <c r="V22" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>78</v>
       </c>
@@ -4394,8 +4905,19 @@
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R23" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S23" s="1"/>
+      <c r="T23" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U23" s="1"/>
+      <c r="V23" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>82</v>
       </c>
@@ -4434,8 +4956,19 @@
       <c r="Q24" s="1" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R24" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S24" s="1"/>
+      <c r="T24" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U24" s="1"/>
+      <c r="V24" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>86</v>
       </c>
@@ -4474,8 +5007,19 @@
       <c r="Q25" s="1" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R25" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S25" s="1"/>
+      <c r="T25" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U25" s="1"/>
+      <c r="V25" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>197</v>
       </c>
@@ -4514,8 +5058,19 @@
       <c r="Q26" s="1" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R26" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S26" s="1"/>
+      <c r="T26" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U26" s="1"/>
+      <c r="V26" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>201</v>
       </c>
@@ -4554,8 +5109,19 @@
       <c r="Q27" s="1" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R27" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S27" s="1"/>
+      <c r="T27" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U27" s="1"/>
+      <c r="V27" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>205</v>
       </c>
@@ -4594,8 +5160,19 @@
       <c r="Q28" s="1" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R28" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S28" s="1"/>
+      <c r="T28" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U28" s="1"/>
+      <c r="V28" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>110</v>
       </c>
@@ -4623,6 +5200,38 @@
       <c r="O29" s="1"/>
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
+      <c r="R29" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="S29" s="1"/>
+      <c r="T29" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="U29" s="1"/>
+      <c r="V29" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
+      <c r="T30" s="1"/>
+      <c r="U30" s="1"/>
+      <c r="V30" s="1"/>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
+      <c r="T31" s="1"/>
+      <c r="U31" s="1"/>
+      <c r="V31" s="1"/>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="R32" s="1"/>
+      <c r="S32" s="1"/>
+      <c r="T32" s="1"/>
+      <c r="U32" s="1"/>
+      <c r="V32" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Phase 2 Part 1: working on hazard unit
</commit_message>
<xml_diff>
--- a/docs/MIPS I ISA.xlsx
+++ b/docs/MIPS I ISA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Digital\SoC\mips_top\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81237FEF-D802-4B88-8411-040CA84ACE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC677F3E-1CE6-414D-9A92-4CD503EAD9BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="463">
   <si>
     <t xml:space="preserve">Opcode </t>
   </si>
@@ -1420,6 +1420,39 @@
   </si>
   <si>
     <t>Execute/Memory/WB 2 Decode Bypass</t>
+  </si>
+  <si>
+    <t>bypass_decode_rs_sel</t>
+  </si>
+  <si>
+    <t>[3 bit] Determine the rs_data in decode stage</t>
+  </si>
+  <si>
+    <t>d_rs_data_regfile</t>
+  </si>
+  <si>
+    <t>bypass_decode_rt_sel</t>
+  </si>
+  <si>
+    <t>[3 bit] Determine the rt_data in decode stage</t>
+  </si>
+  <si>
+    <t>d_rt_data_regfile</t>
+  </si>
+  <si>
+    <t>Used (ALU)</t>
+  </si>
+  <si>
+    <t>Used (SignImm)</t>
+  </si>
+  <si>
+    <t>Used (Multipler Lo)</t>
+  </si>
+  <si>
+    <t>Used (mem_read)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used (ALU) </t>
   </si>
 </sst>
 </file>
@@ -1959,7 +1992,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1313375</xdr:colOff>
+      <xdr:colOff>1308612</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>85923</xdr:rowOff>
     </xdr:to>
@@ -2093,11 +2126,9 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}" name="Table1" displayName="Table1" ref="A1:Y32" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="A1:Y32" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}">
-    <filterColumn colId="4">
+    <filterColumn colId="23">
       <filters>
-        <filter val="[DONE] Phase 1 - Assignement 1"/>
-        <filter val="[DONE] Phase 1 - Assignement 2"/>
-        <filter val="[DONE] Phase 1 - Assignement 3"/>
+        <filter val="Flush f2d register +handle $ra"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -2135,12 +2166,9 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}" name="Table2" displayName="Table2" ref="A1:V29" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
   <autoFilter ref="A1:V29" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}">
-    <filterColumn colId="4">
+    <filterColumn colId="20">
       <filters>
-        <filter val="[DONE] Phase 1 - Assignement 1"/>
-        <filter val="[DONE] Phase 1 - Assignement 2"/>
-        <filter val="[DONE] Phase 1 - Assignement 2 [Not Synthesised]"/>
-        <filter val="[DONE] Phase 1 - Assignement 3"/>
+        <filter val="Flush f2d register +handle $ra"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -2476,6 +2504,8 @@
     <col min="15" max="15" width="16" customWidth="1"/>
     <col min="16" max="16" width="17.33203125" customWidth="1"/>
     <col min="17" max="20" width="8.88671875" customWidth="1"/>
+    <col min="21" max="21" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="25.44140625" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="33.44140625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="11" bestFit="1" customWidth="1"/>
@@ -2585,7 +2615,7 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
     </row>
-    <row r="3" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>90</v>
       </c>
@@ -2639,7 +2669,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -2711,7 +2741,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -2756,7 +2786,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
@@ -2804,7 +2834,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
@@ -2852,7 +2882,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
@@ -2900,7 +2930,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>32</v>
       </c>
@@ -2945,7 +2975,7 @@
       <c r="S10" s="1"/>
       <c r="T10" s="1"/>
       <c r="U10" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="W10" t="s">
         <v>443</v>
@@ -2954,7 +2984,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>36</v>
       </c>
@@ -2978,7 +3008,7 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
       <c r="U11" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="W11" t="s">
         <v>443</v>
@@ -2987,7 +3017,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>39</v>
       </c>
@@ -3032,7 +3062,7 @@
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
       <c r="U12" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="W12" t="s">
         <v>443</v>
@@ -3041,7 +3071,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>43</v>
       </c>
@@ -3062,7 +3092,7 @@
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
       <c r="U13" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="W13" t="s">
         <v>443</v>
@@ -3071,7 +3101,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>46</v>
       </c>
@@ -3116,7 +3146,7 @@
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
       <c r="U14" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="W14" t="s">
         <v>443</v>
@@ -3125,7 +3155,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>50</v>
       </c>
@@ -3170,7 +3200,7 @@
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
       <c r="U15" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="W15" t="s">
         <v>443</v>
@@ -3179,7 +3209,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>54</v>
       </c>
@@ -3224,7 +3254,7 @@
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
       <c r="U16" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="W16" t="s">
         <v>443</v>
@@ -3233,7 +3263,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>58</v>
       </c>
@@ -3266,7 +3296,7 @@
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
       <c r="U17" t="s">
-        <v>442</v>
+        <v>459</v>
       </c>
       <c r="W17" t="s">
         <v>443</v>
@@ -3334,7 +3364,7 @@
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
     </row>
-    <row r="21" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:25" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>97</v>
       </c>
@@ -3364,7 +3394,7 @@
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>
       <c r="U21" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="W21" t="s">
         <v>443</v>
@@ -3373,7 +3403,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>70</v>
       </c>
@@ -3415,7 +3445,7 @@
       <c r="S22" s="1"/>
       <c r="T22" s="1"/>
       <c r="V22" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="W22" t="s">
         <v>443</v>
@@ -3424,7 +3454,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>74</v>
       </c>
@@ -3466,7 +3496,7 @@
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
       <c r="V23" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="W23" t="s">
         <v>443</v>
@@ -3475,7 +3505,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>78</v>
       </c>
@@ -3514,7 +3544,7 @@
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
       <c r="V24" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="W24" t="s">
         <v>443</v>
@@ -3523,7 +3553,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>82</v>
       </c>
@@ -3565,7 +3595,7 @@
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
       <c r="V25" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="W25" t="s">
         <v>443</v>
@@ -3574,7 +3604,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>86</v>
       </c>
@@ -3616,7 +3646,7 @@
       <c r="S26" s="1"/>
       <c r="T26" s="1"/>
       <c r="V26" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="W26" t="s">
         <v>443</v>
@@ -3667,7 +3697,7 @@
       <c r="S28" s="1"/>
       <c r="T28" s="1"/>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>110</v>
       </c>
@@ -3706,7 +3736,7 @@
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
       <c r="V29" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="Y29" t="s">
         <v>446</v>
@@ -3797,6 +3827,7 @@
     <col min="15" max="15" width="11.77734375" customWidth="1"/>
     <col min="16" max="16" width="12.109375" customWidth="1"/>
     <col min="17" max="17" width="20.109375" customWidth="1"/>
+    <col min="18" max="18" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="25.88671875" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="26.77734375" bestFit="1" customWidth="1"/>
   </cols>
@@ -3869,7 +3900,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -3908,7 +3939,7 @@
         <v>316</v>
       </c>
       <c r="R2" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="T2" t="s">
         <v>443</v>
@@ -3917,7 +3948,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -3956,7 +3987,7 @@
         <v>317</v>
       </c>
       <c r="R3" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="T3" t="s">
         <v>443</v>
@@ -3965,7 +3996,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -4004,7 +4035,7 @@
         <v>318</v>
       </c>
       <c r="R4" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="T4" t="s">
         <v>443</v>
@@ -4013,7 +4044,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -4052,7 +4083,7 @@
         <v>319</v>
       </c>
       <c r="R5" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="T5" t="s">
         <v>443</v>
@@ -4061,7 +4092,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -4100,7 +4131,7 @@
         <v>320</v>
       </c>
       <c r="R6" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="T6" t="s">
         <v>443</v>
@@ -4109,7 +4140,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -4148,7 +4179,7 @@
         <v>321</v>
       </c>
       <c r="R7" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="T7" t="s">
         <v>443</v>
@@ -4157,7 +4188,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>32</v>
       </c>
@@ -4331,7 +4362,7 @@
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>152</v>
       </c>
@@ -4389,7 +4420,7 @@
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>63</v>
       </c>
@@ -4447,7 +4478,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>159</v>
       </c>
@@ -4505,7 +4536,7 @@
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>163</v>
       </c>
@@ -4563,7 +4594,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>167</v>
       </c>
@@ -4645,7 +4676,7 @@
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
     </row>
-    <row r="18" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>174</v>
       </c>
@@ -4727,7 +4758,7 @@
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>70</v>
       </c>
@@ -4769,7 +4800,7 @@
         <v>309</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S20" s="1"/>
       <c r="T20" s="1" t="s">
@@ -4780,7 +4811,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>74</v>
       </c>
@@ -4811,7 +4842,7 @@
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
       <c r="R21" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S21" s="1"/>
       <c r="T21" s="1" t="s">
@@ -4822,7 +4853,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>185</v>
       </c>
@@ -4864,7 +4895,7 @@
         <v>310</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S22" s="1"/>
       <c r="T22" s="1" t="s">
@@ -4875,7 +4906,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>78</v>
       </c>
@@ -4906,7 +4937,7 @@
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
       <c r="R23" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S23" s="1"/>
       <c r="T23" s="1" t="s">
@@ -4917,7 +4948,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>82</v>
       </c>
@@ -4957,7 +4988,7 @@
         <v>311</v>
       </c>
       <c r="R24" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S24" s="1"/>
       <c r="T24" s="1" t="s">
@@ -4968,7 +4999,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>86</v>
       </c>
@@ -5008,7 +5039,7 @@
         <v>312</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S25" s="1"/>
       <c r="T25" s="1" t="s">
@@ -5019,7 +5050,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>197</v>
       </c>
@@ -5059,7 +5090,7 @@
         <v>314</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S26" s="1"/>
       <c r="T26" s="1" t="s">
@@ -5070,7 +5101,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>201</v>
       </c>
@@ -5110,7 +5141,7 @@
         <v>315</v>
       </c>
       <c r="R27" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S27" s="1"/>
       <c r="T27" s="1" t="s">
@@ -5121,7 +5152,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>205</v>
       </c>
@@ -5161,7 +5192,7 @@
         <v>313</v>
       </c>
       <c r="R28" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S28" s="1"/>
       <c r="T28" s="1" t="s">
@@ -5172,7 +5203,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>110</v>
       </c>
@@ -5201,7 +5232,7 @@
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
       <c r="R29" s="1" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="S29" s="1"/>
       <c r="T29" s="1" t="s">
@@ -5245,10 +5276,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC34BEC-07EC-4D50-AC0B-49504B180A90}">
-  <dimension ref="A1:B102"/>
+  <dimension ref="A1:B122"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.109375" customWidth="1"/>
     <col min="6" max="6" width="41.6640625" customWidth="1"/>
@@ -5948,6 +5979,108 @@
       </c>
       <c r="B102" t="s">
         <v>433</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104" s="17" t="s">
+        <v>452</v>
+      </c>
+      <c r="B104" s="17" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105">
+        <v>0</v>
+      </c>
+      <c r="B105" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A106">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A107">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A108">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A109">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A110">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A112">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A114" s="17" t="s">
+        <v>455</v>
+      </c>
+      <c r="B114" s="17" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115">
+        <v>0</v>
+      </c>
+      <c r="B115" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A118">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A119">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A120">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A121">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A122">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phase 2 Part 1: Environment Cleanup is complete
</commit_message>
<xml_diff>
--- a/docs/MIPS I ISA.xlsx
+++ b/docs/MIPS I ISA.xlsx
@@ -21,6 +21,7 @@
     <sheet name="Verification Plan" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1709,150 +1710,6 @@
   </cellStyles>
   <dxfs count="59">
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
@@ -1963,6 +1820,150 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2124,7 +2125,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}" name="Table1" displayName="Table1" ref="A1:Y32" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}" name="Table1" displayName="Table1" ref="A1:Y32" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="A1:Y32" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}">
     <filterColumn colId="23">
       <filters>
@@ -2133,38 +2134,38 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{6F141741-2C51-4220-AFC7-E5871EC6CD8F}" name="Opcode " dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{94AD8F24-8B7B-488A-B2A5-515BD41E7F08}" name="Name " dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{F54D0553-BC6A-48B5-9E0F-A0BF767398A8}" name="Description " dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{E6BC317F-8DC6-4A10-97A3-062D0A6033C4}" name="Operation" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{4C0751C6-22DE-48F3-A333-C0824C0F0EFD}" name="Comments" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{599EA1B7-5FC4-4650-9D00-5A65D2D76FD2}" name="ReWrite" dataDxfId="40"/>
-    <tableColumn id="7" xr3:uid="{FADF9286-B678-4102-91DC-1ADDBF050E85}" name="RegDst" dataDxfId="39"/>
-    <tableColumn id="8" xr3:uid="{0CF239B5-36C7-4DBC-8249-487AE1E5F5A5}" name="AluSrc" dataDxfId="38"/>
-    <tableColumn id="9" xr3:uid="{1BC2ABDC-0C79-4111-A3DE-6C63C94FA5D5}" name="MemWrite" dataDxfId="37"/>
-    <tableColumn id="10" xr3:uid="{0153894A-151B-41AD-B603-B7BF55EEBE9C}" name="Write_back_sel" dataDxfId="36"/>
-    <tableColumn id="11" xr3:uid="{C68ADF0D-C375-4115-93EF-CD4021B0BD3E}" name="AluOp" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{6F141741-2C51-4220-AFC7-E5871EC6CD8F}" name="Opcode " dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{94AD8F24-8B7B-488A-B2A5-515BD41E7F08}" name="Name " dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{F54D0553-BC6A-48B5-9E0F-A0BF767398A8}" name="Description " dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{E6BC317F-8DC6-4A10-97A3-062D0A6033C4}" name="Operation" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{4C0751C6-22DE-48F3-A333-C0824C0F0EFD}" name="Comments" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{599EA1B7-5FC4-4650-9D00-5A65D2D76FD2}" name="ReWrite" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{FADF9286-B678-4102-91DC-1ADDBF050E85}" name="RegDst" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{0CF239B5-36C7-4DBC-8249-487AE1E5F5A5}" name="AluSrc" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{1BC2ABDC-0C79-4111-A3DE-6C63C94FA5D5}" name="MemWrite" dataDxfId="24"/>
+    <tableColumn id="10" xr3:uid="{0153894A-151B-41AD-B603-B7BF55EEBE9C}" name="Write_back_sel" dataDxfId="23"/>
+    <tableColumn id="11" xr3:uid="{C68ADF0D-C375-4115-93EF-CD4021B0BD3E}" name="AluOp" dataDxfId="22"/>
     <tableColumn id="20" xr3:uid="{4B7A4639-28F0-4297-B746-1FB610AB5BC3}" name="AluOp_immediate"/>
     <tableColumn id="18" xr3:uid="{8FFAE8F4-2929-40DB-8CDB-B6B62F5A5B1D}" name="wb_se_select"/>
     <tableColumn id="21" xr3:uid="{83AF33B5-363D-492B-8E5C-C63E2DB98A90}" name="se_select"/>
-    <tableColumn id="12" xr3:uid="{F1D4D373-D3C9-4BF4-9941-4766A9F778CF}" name="Overflow Mask" dataDxfId="34"/>
-    <tableColumn id="13" xr3:uid="{E4CE9616-85BB-465A-8E96-A5EC285FC9E7}" name="PC Src" dataDxfId="33"/>
-    <tableColumn id="14" xr3:uid="{65386F80-7AF9-4CF2-BDE0-29D2094B577A}" name="hi_write" dataDxfId="32"/>
-    <tableColumn id="15" xr3:uid="{FA558C62-1F5B-4CE1-A1DE-149585FE9142}" name="lo_write" dataDxfId="31"/>
-    <tableColumn id="16" xr3:uid="{D1B88377-9E5B-4D25-B01D-35C955F02CF0}" name="hi_select" dataDxfId="30"/>
-    <tableColumn id="17" xr3:uid="{F28DE1E5-F9D3-44FC-AA82-3DBE9E42FAEC}" name="lo_select" dataDxfId="29"/>
-    <tableColumn id="19" xr3:uid="{390BDAAC-6935-4C11-B3D2-24BF002BA904}" name="Execute " dataDxfId="4"/>
-    <tableColumn id="22" xr3:uid="{D9F15294-478E-42F4-BA78-FA287163229E}" name="Memory" dataDxfId="3"/>
-    <tableColumn id="23" xr3:uid="{FF7FA640-5713-4F28-BCA2-FA75BE7EA342}" name="Writeback" dataDxfId="2"/>
-    <tableColumn id="24" xr3:uid="{959B7067-1726-4B40-95D5-DFB8C3638973}" name="Control Hazard" dataDxfId="1"/>
-    <tableColumn id="25" xr3:uid="{D22C01B1-0878-4B6A-95B0-C87FF0D4AE43}" name="Data Hazard" dataDxfId="0"/>
+    <tableColumn id="12" xr3:uid="{F1D4D373-D3C9-4BF4-9941-4766A9F778CF}" name="Overflow Mask" dataDxfId="21"/>
+    <tableColumn id="13" xr3:uid="{E4CE9616-85BB-465A-8E96-A5EC285FC9E7}" name="PC Src" dataDxfId="20"/>
+    <tableColumn id="14" xr3:uid="{65386F80-7AF9-4CF2-BDE0-29D2094B577A}" name="hi_write" dataDxfId="19"/>
+    <tableColumn id="15" xr3:uid="{FA558C62-1F5B-4CE1-A1DE-149585FE9142}" name="lo_write" dataDxfId="18"/>
+    <tableColumn id="16" xr3:uid="{D1B88377-9E5B-4D25-B01D-35C955F02CF0}" name="hi_select" dataDxfId="17"/>
+    <tableColumn id="17" xr3:uid="{F28DE1E5-F9D3-44FC-AA82-3DBE9E42FAEC}" name="lo_select" dataDxfId="16"/>
+    <tableColumn id="19" xr3:uid="{390BDAAC-6935-4C11-B3D2-24BF002BA904}" name="Execute " dataDxfId="15"/>
+    <tableColumn id="22" xr3:uid="{D9F15294-478E-42F4-BA78-FA287163229E}" name="Memory" dataDxfId="14"/>
+    <tableColumn id="23" xr3:uid="{FF7FA640-5713-4F28-BCA2-FA75BE7EA342}" name="Writeback" dataDxfId="13"/>
+    <tableColumn id="24" xr3:uid="{959B7067-1726-4B40-95D5-DFB8C3638973}" name="Control Hazard" dataDxfId="12"/>
+    <tableColumn id="25" xr3:uid="{D22C01B1-0878-4B6A-95B0-C87FF0D4AE43}" name="Data Hazard" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}" name="Table2" displayName="Table2" ref="A1:V29" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}" name="Table2" displayName="Table2" ref="A1:V29" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="A1:V29" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}">
     <filterColumn colId="20">
       <filters>
@@ -2173,53 +2174,53 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="22">
-    <tableColumn id="1" xr3:uid="{CD4B495D-BEBD-4687-9E48-13E31F1A5458}" name="Funct " dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{E7F73B4A-D35B-4A89-BCB0-DFA47DFF3033}" name="Name " dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{87DDDCA8-8D3D-45D9-835E-8024A1DEE513}" name="Description " dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{1A74FB59-C961-44A8-A91C-BB37DF112620}" name="Operation" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{916118AB-C4A0-47F3-87B2-8F2F5A96272D}" name="Comments" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{A9D2244B-08FE-4D9B-B85E-939B8D1FCDA2}" name="ReWrite" dataDxfId="21"/>
-    <tableColumn id="13" xr3:uid="{0B472683-72C5-483F-A1F5-D2FDA9886CAC}" name="RegDst" dataDxfId="20"/>
-    <tableColumn id="14" xr3:uid="{B2AB814A-4427-483D-92F7-16C5C8659619}" name="AluSrc" dataDxfId="19"/>
-    <tableColumn id="16" xr3:uid="{D1503AC1-DA6F-431E-86E3-3CD8BAD27F47}" name="Write_Back_sel" dataDxfId="18"/>
-    <tableColumn id="17" xr3:uid="{03DAA7C4-6940-4324-93F3-3F703363AC9E}" name="AluOp" dataDxfId="17"/>
-    <tableColumn id="18" xr3:uid="{B4769B34-7E40-48A1-81CF-AF31CD8F17DF}" name="overflow Mask" dataDxfId="16"/>
-    <tableColumn id="19" xr3:uid="{804568FB-85BF-40E3-B057-9BD0161489CA}" name="PCsrc" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{E7BF6538-000F-4221-BEAF-1B1069F544DF}" name="hi_write" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{EB15F963-101B-4FD6-8C35-479C603DBCE6}" name="lo_write" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{B96C025F-6BE7-4A63-8A28-B9122951D973}" name="hi_select" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{585ED190-3E47-430F-B835-ADAC4874BFFD}" name="lo_select" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{2C2B3870-9B9E-459D-B78A-1F301F881E15}" name="AluControl" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{6F7BBD8D-8BB1-43BB-92F8-BA3005A4DF49}" name="Execute " dataDxfId="9"/>
-    <tableColumn id="15" xr3:uid="{1FF65792-45A2-40C0-8B41-9DB94001A189}" name="Memory" dataDxfId="8"/>
-    <tableColumn id="20" xr3:uid="{5E12103B-CEA1-489E-B3A0-711EF959001C}" name="Writeback" dataDxfId="7"/>
-    <tableColumn id="21" xr3:uid="{9DFD91F3-7DF9-46A0-9289-D1240309AAF3}" name="Control Hazard" dataDxfId="6"/>
-    <tableColumn id="22" xr3:uid="{8AA0B39B-B245-4D8F-97FF-7A4FD54C1E29}" name="Data Hazard" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{CD4B495D-BEBD-4687-9E48-13E31F1A5458}" name="Funct " dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{E7F73B4A-D35B-4A89-BCB0-DFA47DFF3033}" name="Name " dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{87DDDCA8-8D3D-45D9-835E-8024A1DEE513}" name="Description " dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{1A74FB59-C961-44A8-A91C-BB37DF112620}" name="Operation" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{916118AB-C4A0-47F3-87B2-8F2F5A96272D}" name="Comments" dataDxfId="52"/>
+    <tableColumn id="12" xr3:uid="{A9D2244B-08FE-4D9B-B85E-939B8D1FCDA2}" name="ReWrite" dataDxfId="51"/>
+    <tableColumn id="13" xr3:uid="{0B472683-72C5-483F-A1F5-D2FDA9886CAC}" name="RegDst" dataDxfId="50"/>
+    <tableColumn id="14" xr3:uid="{B2AB814A-4427-483D-92F7-16C5C8659619}" name="AluSrc" dataDxfId="49"/>
+    <tableColumn id="16" xr3:uid="{D1503AC1-DA6F-431E-86E3-3CD8BAD27F47}" name="Write_Back_sel" dataDxfId="48"/>
+    <tableColumn id="17" xr3:uid="{03DAA7C4-6940-4324-93F3-3F703363AC9E}" name="AluOp" dataDxfId="47"/>
+    <tableColumn id="18" xr3:uid="{B4769B34-7E40-48A1-81CF-AF31CD8F17DF}" name="overflow Mask" dataDxfId="46"/>
+    <tableColumn id="19" xr3:uid="{804568FB-85BF-40E3-B057-9BD0161489CA}" name="PCsrc" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{E7BF6538-000F-4221-BEAF-1B1069F544DF}" name="hi_write" dataDxfId="44"/>
+    <tableColumn id="9" xr3:uid="{EB15F963-101B-4FD6-8C35-479C603DBCE6}" name="lo_write" dataDxfId="43"/>
+    <tableColumn id="10" xr3:uid="{B96C025F-6BE7-4A63-8A28-B9122951D973}" name="hi_select" dataDxfId="42"/>
+    <tableColumn id="11" xr3:uid="{585ED190-3E47-430F-B835-ADAC4874BFFD}" name="lo_select" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{2C2B3870-9B9E-459D-B78A-1F301F881E15}" name="AluControl" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{6F7BBD8D-8BB1-43BB-92F8-BA3005A4DF49}" name="Execute " dataDxfId="39"/>
+    <tableColumn id="15" xr3:uid="{1FF65792-45A2-40C0-8B41-9DB94001A189}" name="Memory" dataDxfId="38"/>
+    <tableColumn id="20" xr3:uid="{5E12103B-CEA1-489E-B3A0-711EF959001C}" name="Writeback" dataDxfId="37"/>
+    <tableColumn id="21" xr3:uid="{9DFD91F3-7DF9-46A0-9289-D1240309AAF3}" name="Control Hazard" dataDxfId="36"/>
+    <tableColumn id="22" xr3:uid="{8AA0B39B-B245-4D8F-97FF-7A4FD54C1E29}" name="Data Hazard" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D53E060B-7B9B-43C9-B6C3-0ADAD9EBE1D7}" name="Table3" displayName="Table3" ref="A1:D10" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{D53E060B-7B9B-43C9-B6C3-0ADAD9EBE1D7}" name="Table3" displayName="Table3" ref="A1:D10" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:D10" xr:uid="{D53E060B-7B9B-43C9-B6C3-0ADAD9EBE1D7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{9277D667-9F6C-4B1A-9BD6-8F4F09DC6FCC}" name="Funct " dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{44121D79-0FB6-4BA0-822D-A22356C92E27}" name="Name " dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{9FFE180B-8031-4716-9450-AF517E4275A8}" name="Description " dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{700AEF16-A70F-499B-87D2-32234302488E}" name="Operation" dataDxfId="53"/>
+    <tableColumn id="1" xr3:uid="{9277D667-9F6C-4B1A-9BD6-8F4F09DC6FCC}" name="Funct " dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{44121D79-0FB6-4BA0-822D-A22356C92E27}" name="Name " dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{9FFE180B-8031-4716-9450-AF517E4275A8}" name="Description " dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{700AEF16-A70F-499B-87D2-32234302488E}" name="Operation" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4ED1B589-2AD4-4E0A-A923-4EE6DF5E917F}" name="Table4" displayName="Table4" ref="A1:C11" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4ED1B589-2AD4-4E0A-A923-4EE6DF5E917F}" name="Table4" displayName="Table4" ref="A1:C11" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="A1:C11" xr:uid="{4ED1B589-2AD4-4E0A-A923-4EE6DF5E917F}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{54084E4B-9E28-4AC8-AF1B-3C8B1A6C439F}" name="Test #" dataDxfId="50"/>
-    <tableColumn id="2" xr3:uid="{BD73A61D-1FF1-4476-B2A3-42E28CFEB520}" name="Function" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{89ABFDA6-6F2C-4281-BB66-65F42B941C05}" name="Description" dataDxfId="48"/>
+    <tableColumn id="1" xr3:uid="{54084E4B-9E28-4AC8-AF1B-3C8B1A6C439F}" name="Test #" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{BD73A61D-1FF1-4476-B2A3-42E28CFEB520}" name="Function" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{89ABFDA6-6F2C-4281-BB66-65F42B941C05}" name="Description" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Phase 1 Part 1: Test 1 is Passed
</commit_message>
<xml_diff>
--- a/docs/MIPS I ISA.xlsx
+++ b/docs/MIPS I ISA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Digital\SoC\mips_top\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC677F3E-1CE6-414D-9A92-4CD503EAD9BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20A00054-AB9C-4D67-ADF7-14304FFD01B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main ISA" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="Verification Plan" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -31,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="481">
   <si>
     <t xml:space="preserve">Opcode </t>
   </si>
@@ -1454,6 +1453,60 @@
   </si>
   <si>
     <t xml:space="preserve">Used (ALU) </t>
+  </si>
+  <si>
+    <t>m_alu_result</t>
+  </si>
+  <si>
+    <t>m_mult_lo</t>
+  </si>
+  <si>
+    <t>m_se_imm</t>
+  </si>
+  <si>
+    <t>wb_mem_data</t>
+  </si>
+  <si>
+    <t>wb_data</t>
+  </si>
+  <si>
+    <t>b0</t>
+  </si>
+  <si>
+    <t>bypass_execute_rs_sel</t>
+  </si>
+  <si>
+    <t>bypass_execute_rt_sel</t>
+  </si>
+  <si>
+    <t>[3 bit] Determine the rs_data in Execute stage</t>
+  </si>
+  <si>
+    <t>[3 bit] Determine the rt_data in Execute stage</t>
+  </si>
+  <si>
+    <t>bypass_mem_rs_sel</t>
+  </si>
+  <si>
+    <t>bypass_mem_rt_sel</t>
+  </si>
+  <si>
+    <t>[2 bit] Determine the rs_data in Memory stage</t>
+  </si>
+  <si>
+    <t>e_rt_data_d2e</t>
+  </si>
+  <si>
+    <t>e_rs_data_d2e</t>
+  </si>
+  <si>
+    <t>m_rs_data_e2m</t>
+  </si>
+  <si>
+    <t>[2 bit] Determine the rt_data in Memory stage</t>
+  </si>
+  <si>
+    <t>m_rt_data_e2m</t>
   </si>
 </sst>
 </file>
@@ -1640,7 +1693,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1704,6 +1757,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2088,7 +2144,7 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>900732</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>167151</xdr:rowOff>
+      <xdr:rowOff>167152</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2126,13 +2182,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}" name="Table1" displayName="Table1" ref="A1:Y32" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
-  <autoFilter ref="A1:Y32" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}">
-    <filterColumn colId="23">
-      <filters>
-        <filter val="Flush f2d register +handle $ra"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:Y32" xr:uid="{0D33F033-7401-4F1F-8987-FB63CD7DF6BC}"/>
   <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{6F141741-2C51-4220-AFC7-E5871EC6CD8F}" name="Opcode " dataDxfId="32"/>
     <tableColumn id="2" xr3:uid="{94AD8F24-8B7B-488A-B2A5-515BD41E7F08}" name="Name " dataDxfId="31"/>
@@ -2166,13 +2216,7 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}" name="Table2" displayName="Table2" ref="A1:V29" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
-  <autoFilter ref="A1:V29" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}">
-    <filterColumn colId="20">
-      <filters>
-        <filter val="Flush f2d register +handle $ra"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:V29" xr:uid="{151E0FC9-74A1-4492-82A5-A6974E379F5E}"/>
   <tableColumns count="22">
     <tableColumn id="1" xr3:uid="{CD4B495D-BEBD-4687-9E48-13E31F1A5458}" name="Funct " dataDxfId="56"/>
     <tableColumn id="2" xr3:uid="{E7F73B4A-D35B-4A89-BCB0-DFA47DFF3033}" name="Name " dataDxfId="55"/>
@@ -2597,7 +2641,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="2" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2616,7 +2660,7 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
     </row>
-    <row r="3" spans="1:28" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>90</v>
       </c>
@@ -2670,7 +2714,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="4" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -2742,7 +2786,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="6" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -2787,7 +2831,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="7" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
@@ -2835,7 +2879,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="8" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
@@ -2883,7 +2927,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="9" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
@@ -2931,7 +2975,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="10" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>32</v>
       </c>
@@ -2985,7 +3029,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="11" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>36</v>
       </c>
@@ -3018,7 +3062,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="12" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>39</v>
       </c>
@@ -3072,7 +3116,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="13" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>43</v>
       </c>
@@ -3102,7 +3146,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="14" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>46</v>
       </c>
@@ -3156,7 +3200,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="15" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>50</v>
       </c>
@@ -3210,7 +3254,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="16" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>54</v>
       </c>
@@ -3264,7 +3308,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="17" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>58</v>
       </c>
@@ -3306,7 +3350,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>94</v>
       </c>
@@ -3327,7 +3371,7 @@
       <c r="S18" s="1"/>
       <c r="T18" s="1"/>
     </row>
-    <row r="19" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>63</v>
       </c>
@@ -3346,7 +3390,7 @@
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
     </row>
-    <row r="20" spans="1:25" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>98</v>
       </c>
@@ -3365,7 +3409,7 @@
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
     </row>
-    <row r="21" spans="1:25" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:25" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>97</v>
       </c>
@@ -3404,7 +3448,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="22" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>70</v>
       </c>
@@ -3455,7 +3499,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="23" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>74</v>
       </c>
@@ -3506,7 +3550,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="24" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>78</v>
       </c>
@@ -3554,7 +3598,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="25" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>82</v>
       </c>
@@ -3605,7 +3649,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="26" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>86</v>
       </c>
@@ -3656,7 +3700,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="27" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>102</v>
       </c>
@@ -3677,7 +3721,7 @@
       <c r="S27" s="1"/>
       <c r="T27" s="1"/>
     </row>
-    <row r="28" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>106</v>
       </c>
@@ -3698,7 +3742,7 @@
       <c r="S28" s="1"/>
       <c r="T28" s="1"/>
     </row>
-    <row r="29" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>110</v>
       </c>
@@ -3743,7 +3787,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="30" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>114</v>
       </c>
@@ -3762,7 +3806,7 @@
       <c r="S30" s="1"/>
       <c r="T30" s="1"/>
     </row>
-    <row r="31" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>118</v>
       </c>
@@ -3781,7 +3825,7 @@
       <c r="S31" s="1"/>
       <c r="T31" s="1"/>
     </row>
-    <row r="32" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -3901,7 +3945,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="2" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -3949,7 +3993,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="3" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -3997,7 +4041,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="4" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -4045,7 +4089,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="5" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -4093,7 +4137,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="6" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -4141,7 +4185,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="7" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -4189,7 +4233,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="8" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>32</v>
       </c>
@@ -4295,7 +4339,7 @@
       </c>
       <c r="V9" s="1"/>
     </row>
-    <row r="10" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>145</v>
       </c>
@@ -4329,7 +4373,7 @@
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
     </row>
-    <row r="11" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>149</v>
       </c>
@@ -4363,7 +4407,7 @@
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
     </row>
-    <row r="12" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>152</v>
       </c>
@@ -4421,7 +4465,7 @@
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
     </row>
-    <row r="13" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>63</v>
       </c>
@@ -4479,7 +4523,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="14" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>159</v>
       </c>
@@ -4537,7 +4581,7 @@
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>163</v>
       </c>
@@ -4595,7 +4639,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>167</v>
       </c>
@@ -4645,7 +4689,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="17" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>171</v>
       </c>
@@ -4677,7 +4721,7 @@
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
     </row>
-    <row r="18" spans="1:22" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>174</v>
       </c>
@@ -4727,7 +4771,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>177</v>
       </c>
@@ -4759,7 +4803,7 @@
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
     </row>
-    <row r="20" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>70</v>
       </c>
@@ -4812,7 +4856,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="21" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>74</v>
       </c>
@@ -4854,7 +4898,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="22" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>185</v>
       </c>
@@ -4907,7 +4951,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="23" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>78</v>
       </c>
@@ -4949,7 +4993,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="24" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>82</v>
       </c>
@@ -5000,7 +5044,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="25" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>86</v>
       </c>
@@ -5051,7 +5095,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="26" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>197</v>
       </c>
@@ -5102,7 +5146,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="27" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>201</v>
       </c>
@@ -5153,7 +5197,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="28" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>205</v>
       </c>
@@ -5204,7 +5248,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="29" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>110</v>
       </c>
@@ -5277,7 +5321,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC34BEC-07EC-4D50-AC0B-49504B180A90}">
-  <dimension ref="A1:B122"/>
+  <dimension ref="A1:B162"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -6002,36 +6046,57 @@
       <c r="A106">
         <v>1</v>
       </c>
+      <c r="B106" t="s">
+        <v>463</v>
+      </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>2</v>
       </c>
+      <c r="B107" t="s">
+        <v>464</v>
+      </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>3</v>
       </c>
+      <c r="B108" t="s">
+        <v>465</v>
+      </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>4</v>
       </c>
+      <c r="B109" t="s">
+        <v>466</v>
+      </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>5</v>
       </c>
+      <c r="B110" t="s">
+        <v>467</v>
+      </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>6</v>
       </c>
+      <c r="B111" s="23" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>7</v>
       </c>
+      <c r="B112" s="23" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" s="17" t="s">
@@ -6053,36 +6118,313 @@
       <c r="A116">
         <v>1</v>
       </c>
+      <c r="B116" t="s">
+        <v>463</v>
+      </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>2</v>
       </c>
+      <c r="B117" t="s">
+        <v>464</v>
+      </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>3</v>
       </c>
+      <c r="B118" t="s">
+        <v>465</v>
+      </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>4</v>
       </c>
+      <c r="B119" t="s">
+        <v>466</v>
+      </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>5</v>
       </c>
+      <c r="B120" t="s">
+        <v>467</v>
+      </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>6</v>
       </c>
+      <c r="B121" s="23" t="s">
+        <v>468</v>
+      </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>7</v>
       </c>
+      <c r="B122" s="23" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A124" s="17" t="s">
+        <v>469</v>
+      </c>
+      <c r="B124" s="17" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A125">
+        <v>0</v>
+      </c>
+      <c r="B125" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A126">
+        <v>1</v>
+      </c>
+      <c r="B126" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A127">
+        <v>2</v>
+      </c>
+      <c r="B127" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A128">
+        <v>3</v>
+      </c>
+      <c r="B128" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A129">
+        <v>4</v>
+      </c>
+      <c r="B129" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A130">
+        <v>5</v>
+      </c>
+      <c r="B130" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A131">
+        <v>6</v>
+      </c>
+      <c r="B131" s="23" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A132">
+        <v>7</v>
+      </c>
+      <c r="B132" s="23" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A134" s="17" t="s">
+        <v>470</v>
+      </c>
+      <c r="B134" s="17" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A135">
+        <v>0</v>
+      </c>
+      <c r="B135" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A136">
+        <v>1</v>
+      </c>
+      <c r="B136" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A137">
+        <v>2</v>
+      </c>
+      <c r="B137" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A138">
+        <v>3</v>
+      </c>
+      <c r="B138" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A139">
+        <v>4</v>
+      </c>
+      <c r="B139" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A140">
+        <v>5</v>
+      </c>
+      <c r="B140" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A141">
+        <v>6</v>
+      </c>
+      <c r="B141" s="23" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A142">
+        <v>7</v>
+      </c>
+      <c r="B142" s="23" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A144" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="B144" s="17" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A145">
+        <v>0</v>
+      </c>
+      <c r="B145" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A146">
+        <v>1</v>
+      </c>
+      <c r="B146" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A147">
+        <v>2</v>
+      </c>
+      <c r="B147" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A148">
+        <v>3</v>
+      </c>
+      <c r="B148" s="23" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A150" s="17" t="s">
+        <v>474</v>
+      </c>
+      <c r="B150" s="17" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A151">
+        <v>0</v>
+      </c>
+      <c r="B151" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A152">
+        <v>1</v>
+      </c>
+      <c r="B152" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A153">
+        <v>2</v>
+      </c>
+      <c r="B153" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A154">
+        <v>3</v>
+      </c>
+      <c r="B154" s="23" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A155" s="24"/>
+      <c r="B155" s="24"/>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A156" s="24"/>
+      <c r="B156" s="24"/>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A157" s="24"/>
+      <c r="B157" s="24"/>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A158" s="24"/>
+      <c r="B158" s="24"/>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A159" s="24"/>
+      <c r="B159" s="24"/>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A160" s="24"/>
+      <c r="B160" s="24"/>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A161" s="24"/>
+      <c r="B161" s="25"/>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A162" s="24"/>
+      <c r="B162" s="25"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>